<commit_message>
Modelo e dados CC ajustado HRTN
</commit_message>
<xml_diff>
--- a/results/Cenarios.xlsx
+++ b/results/Cenarios.xlsx
@@ -8,13 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\desk-surgery-center\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8077D525-FA79-4EFB-BD99-450675D3999C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C355EB8-396A-44E8-A5C4-601EEF4D724C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{61E1E10E-7175-41C5-8AB5-C7572230C2F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="55">
   <si>
     <t>CC-1</t>
   </si>
@@ -149,9 +153,6 @@
     <t>Período de simulação (dias)</t>
   </si>
   <si>
-    <t>Custo (R$)</t>
-  </si>
-  <si>
     <t>Cirurgias / dia (pacientes)</t>
   </si>
   <si>
@@ -167,9 +168,6 @@
     <t>1-2-2-1</t>
   </si>
   <si>
-    <t>6-12-6</t>
-  </si>
-  <si>
     <t>Prod Sala1 + Escala</t>
   </si>
   <si>
@@ -186,6 +184,27 @@
   </si>
   <si>
     <t>Sabado + 20%</t>
+  </si>
+  <si>
+    <t>Custo Variável (R$)</t>
+  </si>
+  <si>
+    <t>Custo Fixo (R$)</t>
+  </si>
+  <si>
+    <t>Margem de Contribuição (R$)</t>
+  </si>
+  <si>
+    <t>Profissionais</t>
+  </si>
+  <si>
+    <t>Escala (0-7-19)</t>
+  </si>
+  <si>
+    <t>4-6-4</t>
+  </si>
+  <si>
+    <t>3-8-3</t>
   </si>
 </sst>
 </file>
@@ -195,7 +214,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,6 +251,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -241,12 +275,186 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -255,7 +463,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -283,9 +491,41 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -293,7 +533,18 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -304,6 +555,988 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$32</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Margem de Contribuição (R$)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$C$2:$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>CC-0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>CC-1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>CC-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>CC-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>CC-4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>CC-5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>CC-6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>CC-7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>CC-8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$32:$K$32</c:f>
+              <c:numCache>
+                <c:formatCode>_("R$"* #,##0.00_);_("R$"* \(#,##0.00\);_("R$"* "-"??_);_(@_)</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>2815802.9741303846</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2676610.4741455186</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3350736.7905518059</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5569836.2203911524</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5658752.131839348</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3462769.65880326</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3025862.2743492443</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3638326.6555657741</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4430189.9871105924</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-80A0-4C4D-BEAB-CB2E3945B97F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1081628335"/>
+        <c:axId val="1081628815"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1081628335"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1081628815"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1081628815"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="_(&quot;R$&quot;* #,##0.00_);_(&quot;R$&quot;* \(#,##0.00\);_(&quot;R$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1081628335"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
+  <a:schemeClr val="accent6"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent4"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>765664</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>20516</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1348154</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>96716</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C922B8FD-F1C4-4BA2-19D7-7EF386C44000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="ANÁLISE DAS CONTAS"/>
+      <sheetName val="Δ%CONTAS"/>
+      <sheetName val="PRODUTIVOS"/>
+      <sheetName val="COMPARADO"/>
+      <sheetName val="Resumo"/>
+      <sheetName val="2025 C. Total"/>
+      <sheetName val="2022a MV Soul"/>
+      <sheetName val="Resumo MV2000"/>
+      <sheetName val="Leitos CC MV2000"/>
+      <sheetName val="Gr. de Contas"/>
+      <sheetName val="Maternidade"/>
+      <sheetName val="PS "/>
+      <sheetName val="Matern com C. Cirurgico MV Soul"/>
+      <sheetName val="Clin. Méd."/>
+      <sheetName val="Clín. Cirúrgica"/>
+      <sheetName val="Clin cirur c bloco MV Soul"/>
+      <sheetName val="Custos-BC "/>
+      <sheetName val="Receita"/>
+      <sheetName val="DRE"/>
+      <sheetName val="CTI "/>
+      <sheetName val="Ambulatorio"/>
+      <sheetName val="Comparativo"/>
+      <sheetName val="BD Desp. Financ."/>
+      <sheetName val="BD Desp. Custos"/>
+      <sheetName val="PROCV"/>
+      <sheetName val="BD Produtivos"/>
+      <sheetName val="PRIMARIO E DIRETO"/>
+      <sheetName val="BD Pcte. Dia"/>
+      <sheetName val="Receitas produção"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18">
+        <row r="6">
+          <cell r="H6">
+            <v>1227.6414338377958</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="C15">
+            <v>2062261.4850000001</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25"/>
+      <sheetData sheetId="26"/>
+      <sheetData sheetId="27"/>
+      <sheetData sheetId="28"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -623,20 +1856,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C24F749-DA3C-4527-A1DD-2E2827984C34}">
-  <dimension ref="B2:M32"/>
+  <dimension ref="B2:M34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" customWidth="1"/>
-    <col min="10" max="10" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="21.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.85546875" customWidth="1"/>
+    <col min="11" max="11" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
@@ -681,35 +1914,35 @@
       <c r="B3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="G3" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="H3" s="11" t="s">
+      <c r="J3" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="K3" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="J3" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="K3" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B4" s="9" t="s">
         <v>36</v>
       </c>
@@ -747,7 +1980,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B5" s="9" t="s">
         <v>16</v>
       </c>
@@ -783,7 +2016,7 @@
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C6" s="1">
         <v>14.78</v>
@@ -853,39 +2086,39 @@
       </c>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="F9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="H9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>42</v>
-      </c>
       <c r="J9" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -917,39 +2150,39 @@
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -981,7 +2214,7 @@
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="11" t="s">
         <v>32</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -991,19 +2224,19 @@
         <v>27</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>27</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>27</v>
@@ -1013,7 +2246,7 @@
       </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -1023,19 +2256,19 @@
         <v>27</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>27</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>27</v>
@@ -1045,7 +2278,7 @@
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="11" t="s">
         <v>23</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -1077,7 +2310,7 @@
       </c>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -1109,7 +2342,7 @@
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1141,7 +2374,7 @@
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1183,14 +2416,14 @@
       <c r="K19" s="1"/>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C20" s="4">
-        <v>0.26800000000000002</v>
+        <v>0.3</v>
       </c>
       <c r="D20" s="4">
-        <v>0.27</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="E20" s="4">
         <v>0.34</v>
@@ -1215,14 +2448,14 @@
       </c>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="11" t="s">
         <v>19</v>
       </c>
       <c r="C21" s="4">
-        <v>0.34799999999999998</v>
+        <v>0.31</v>
       </c>
       <c r="D21" s="4">
-        <v>0.34799999999999998</v>
+        <v>0.33</v>
       </c>
       <c r="E21" s="4">
         <v>0.32</v>
@@ -1247,14 +2480,14 @@
       </c>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="4">
-        <v>0.6</v>
+        <v>0.76</v>
       </c>
       <c r="D22" s="4">
-        <v>0.66</v>
+        <v>0.95</v>
       </c>
       <c r="E22" s="4">
         <v>0.72</v>
@@ -1279,7 +2512,7 @@
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="11" t="s">
         <v>21</v>
       </c>
       <c r="C23" s="4">
@@ -1311,11 +2544,11 @@
       </c>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="11" t="s">
         <v>32</v>
       </c>
       <c r="C24" s="4">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
       <c r="D24" s="4">
         <v>0.7</v>
@@ -1343,14 +2576,14 @@
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="11" t="s">
         <v>22</v>
       </c>
       <c r="C25" s="4">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="D25" s="4">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="E25" s="4">
         <v>0.44</v>
@@ -1375,14 +2608,14 @@
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="11" t="s">
         <v>23</v>
       </c>
       <c r="C26" s="4">
-        <v>0.35</v>
+        <v>0.32</v>
       </c>
       <c r="D26" s="4">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="E26" s="4">
         <v>0.35</v>
@@ -1407,14 +2640,14 @@
       </c>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C27" s="4">
-        <v>0.35</v>
+        <v>0.32</v>
       </c>
       <c r="D27" s="4">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="E27" s="4">
         <v>0.35</v>
@@ -1439,7 +2672,7 @@
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="11" t="s">
         <v>25</v>
       </c>
       <c r="C28" s="4">
@@ -1471,14 +2704,14 @@
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C29" s="4">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="D29" s="4">
-        <v>0.4</v>
+        <v>0.37</v>
       </c>
       <c r="E29" s="4">
         <v>0.34</v>
@@ -1507,120 +2740,360 @@
         <v>35</v>
       </c>
       <c r="C30" s="3">
-        <v>797131</v>
+        <f>797131*12</f>
+        <v>9565572</v>
       </c>
       <c r="D30" s="3">
-        <v>1086278</v>
+        <f>961735*12</f>
+        <v>11540820</v>
       </c>
       <c r="E30" s="3">
-        <v>920106</v>
+        <f>920106*12</f>
+        <v>11041272</v>
       </c>
       <c r="F30" s="3">
-        <v>1497778</v>
+        <f>1497778*12</f>
+        <v>17973336</v>
       </c>
       <c r="G30" s="3">
-        <v>1518127</v>
+        <f>1518127*12</f>
+        <v>18217524</v>
       </c>
       <c r="H30" s="3">
-        <v>940098</v>
+        <f>940098*12</f>
+        <v>11281176</v>
       </c>
       <c r="I30" s="3">
-        <v>848126</v>
+        <f>848126*12</f>
+        <v>10177512</v>
       </c>
       <c r="J30" s="3">
-        <v>980987</v>
+        <f>980987*12</f>
+        <v>11771844</v>
       </c>
       <c r="K30" s="3">
-        <v>1179033</v>
+        <f>1179033*12</f>
+        <v>14148396</v>
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="10" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C31" s="3">
-        <v>2518808</v>
+        <f>[1]DRE!$H$6*(C6*C4)*12</f>
+        <v>6749769.0258696154</v>
       </c>
       <c r="D31" s="3">
-        <v>3422522</v>
+        <f>[1]DRE!$H$6*(D6*D4)*12</f>
+        <v>8864209.5258544814</v>
       </c>
       <c r="E31" s="3">
-        <v>2927363</v>
+        <f>[1]DRE!$H$6*(E6*E4)*12</f>
+        <v>7690535.2094481941</v>
       </c>
       <c r="F31" s="3">
-        <v>4740480</v>
+        <f>[1]DRE!$H$6*(F6*F4)*12</f>
+        <v>12403499.779608848</v>
       </c>
       <c r="G31" s="3">
-        <v>4820988</v>
+        <f>[1]DRE!$H$6*(G6*G4)*12</f>
+        <v>12558771.868160652</v>
       </c>
       <c r="H31" s="3">
-        <v>2980816</v>
+        <f>[1]DRE!$H$6*(H6*H4)*12</f>
+        <v>7818406.34119674</v>
       </c>
       <c r="I31" s="3">
-        <v>2701863</v>
+        <f>[1]DRE!$H$6*(I6*I4)*12</f>
+        <v>7151649.7256507557</v>
       </c>
       <c r="J31" s="3">
-        <v>3117765</v>
+        <f>[1]DRE!$H$6*(J6*J4)*12</f>
+        <v>8133517.3444342259</v>
       </c>
       <c r="K31" s="3">
-        <v>3740526</v>
+        <f>[1]DRE!$H$6*(K6*K4)*12</f>
+        <v>9718206.0128894076</v>
       </c>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B32" s="10" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C32" s="3">
         <f>C30-C31</f>
-        <v>-1721677</v>
+        <v>2815802.9741303846</v>
       </c>
       <c r="D32" s="3">
         <f>D30-D31</f>
-        <v>-2336244</v>
+        <v>2676610.4741455186</v>
       </c>
       <c r="E32" s="3">
         <f>E30-E31</f>
-        <v>-2007257</v>
+        <v>3350736.7905518059</v>
       </c>
       <c r="F32" s="3">
-        <f>F30-F31</f>
-        <v>-3242702</v>
+        <f t="shared" ref="F32:K32" si="0">F30-F31</f>
+        <v>5569836.2203911524</v>
       </c>
       <c r="G32" s="3">
-        <f>G30-G31</f>
-        <v>-3302861</v>
+        <f t="shared" si="0"/>
+        <v>5658752.131839348</v>
       </c>
       <c r="H32" s="3">
-        <f>H30-H31</f>
-        <v>-2040718</v>
+        <f t="shared" si="0"/>
+        <v>3462769.65880326</v>
       </c>
       <c r="I32" s="3">
-        <f>I30-I31</f>
-        <v>-1853737</v>
+        <f t="shared" si="0"/>
+        <v>3025862.2743492443</v>
       </c>
       <c r="J32" s="3">
-        <f>J30-J31</f>
-        <v>-2136778</v>
+        <f t="shared" si="0"/>
+        <v>3638326.6555657741</v>
       </c>
       <c r="K32" s="3">
-        <f>K30-K31</f>
-        <v>-2561493</v>
+        <f t="shared" si="0"/>
+        <v>4430189.9871105924</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B33" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="D33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="E33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="F33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="G33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="H33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="I33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="J33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+      <c r="K33" s="3">
+        <f>[1]DRE!$C$15*12</f>
+        <v>24747137.82</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B34" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="3">
+        <f>C30-C31-C33</f>
+        <v>-21931334.845869616</v>
+      </c>
+      <c r="D34" s="3">
+        <f t="shared" ref="D34:K34" si="1">D30-D31-D33</f>
+        <v>-22070527.345854484</v>
+      </c>
+      <c r="E34" s="3">
+        <f t="shared" si="1"/>
+        <v>-21396401.029448196</v>
+      </c>
+      <c r="F34" s="3">
+        <f t="shared" si="1"/>
+        <v>-19177301.599608846</v>
+      </c>
+      <c r="G34" s="3">
+        <f t="shared" si="1"/>
+        <v>-19088385.68816065</v>
+      </c>
+      <c r="H34" s="3">
+        <f t="shared" si="1"/>
+        <v>-21284368.161196738</v>
+      </c>
+      <c r="I34" s="3">
+        <f t="shared" si="1"/>
+        <v>-21721275.545650758</v>
+      </c>
+      <c r="J34" s="3">
+        <f t="shared" si="1"/>
+        <v>-21108811.164434224</v>
+      </c>
+      <c r="K34" s="3">
+        <f t="shared" si="1"/>
+        <v>-20316947.832889408</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="C20:M29">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
+  <conditionalFormatting sqref="C20:K29">
+    <cfRule type="iconSet" priority="2">
+      <iconSet reverse="1">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C30:K34">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D64D93C-DFBB-4BE9-9B73-9315A7CA8EF1}">
+  <dimension ref="B1:D12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="16">
+        <v>1</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="19">
+        <v>2</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="19">
+        <v>10</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="19">
+        <v>1</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="19">
+        <v>5</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="19">
+        <v>5</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="19">
+        <v>2</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="19">
+        <v>2</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="19">
+        <v>1</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="22">
+        <v>2</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>